<commit_message>
feat: bandeja de cliente, parejas v4 y estados en minúsculas
- Estados de 03_coches y 04_parejas en el vocabulario común, en minúsculas
  (pendiente_lectura → sin_auditar, formato_invalido → formato).
- 04_parejas: las 66 parejas propuestas por emparejar_v4.
- 02_extraido/bandeja_cliente: conversiones .md por pareja (los PDF de
  01_entrada/bandeja_cliente quedan fuera, en .gitignore).
- Dashboard y bases con los valores nuevos; esquemas y reglas actualizados.
- Informes del 2026-10-29 (experimento v1/v2, sankey, emparejamiento) y
  petición de permisos y fichas.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/05_generado/peticiones/2026-10-29_permisos_y_fichas.xlsx
+++ b/05_generado/peticiones/2026-10-29_permisos_y_fichas.xlsx
@@ -499,7 +499,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2704MXG</t>
+          <t>2705MXG</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -545,7 +545,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2705MXG</t>
+          <t>2720MWP</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -555,7 +555,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>RENAULT KANGOO FURGON E-TECH 100% ELECTRIC</t>
+          <t>Citroën ë-C3 Eléctrico Max</t>
         </is>
       </c>
       <c r="F3" t="n">
@@ -568,7 +568,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>N1</t>
+          <t>M1</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -591,7 +591,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2720MWP</t>
+          <t>2722MXG</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -601,7 +601,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Citroën ë-C3 Eléctrico Max</t>
+          <t>RENAULT KANGOO FURGON E-TECH 100% ELECTRIC</t>
         </is>
       </c>
       <c r="F4" t="n">
@@ -614,7 +614,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>M1</t>
+          <t>N1</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -637,7 +637,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2722MXG</t>
+          <t>2737MXG</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -683,7 +683,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2737MXG</t>
+          <t>6007MWV</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -693,7 +693,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>RENAULT KANGOO FURGON E-TECH 100% ELECTRIC</t>
+          <t>CITROËN ë-C3 Eléctrico Max</t>
         </is>
       </c>
       <c r="F6" t="n">
@@ -706,7 +706,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>N1</t>
+          <t>M1</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -729,7 +729,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>6007MWV</t>
+          <t>6015MWV</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -775,7 +775,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>6015MWV</t>
+          <t>6029MWV</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -821,7 +821,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>6029MWV</t>
+          <t>6042MWV</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -867,7 +867,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>6042MWV</t>
+          <t>6083MWV</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -877,7 +877,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>CITROËN ë-C3 Eléctrico Max</t>
+          <t>Citroën ë-C3</t>
         </is>
       </c>
       <c r="F10" t="n">
@@ -913,7 +913,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>6083MWV</t>
+          <t>6084MWV</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -923,7 +923,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Citroën ë-C3</t>
+          <t>CITROËN ë-C3 Eléctrico Max</t>
         </is>
       </c>
       <c r="F11" t="n">
@@ -959,7 +959,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>6084MWV</t>
+          <t>6087MWV</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1143,7 +1143,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>6334MXF</t>
+          <t>6102MWV</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1153,7 +1153,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>RENAULT KANGOO FURGON E-TECH 100% ELECTRIC</t>
+          <t>CITROËN ë-C3 Eléctrico Max</t>
         </is>
       </c>
       <c r="F16" t="n">
@@ -1166,7 +1166,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>N1</t>
+          <t>M1</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1189,7 +1189,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>6370MXF</t>
+          <t>6334MXF</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1235,7 +1235,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>9050MWN</t>
+          <t>9049MWN</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1245,7 +1245,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Citroën ë-C3 Eléctrico Max</t>
+          <t>CITROEN Ë-C3 ELÉCTRICO MAX</t>
         </is>
       </c>
       <c r="F18" t="n">
@@ -1263,7 +1263,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>extraccion</t>
+          <t>excel</t>
         </is>
       </c>
       <c r="J18" t="inlineStr"/>
@@ -1281,17 +1281,17 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>4926LMS</t>
+          <t>9050MWN</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Sustituido (baja)</t>
+          <t>Nuevo (alta)</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>PEUGEOT Partner Premium Standard 600kg BlueHDi 100 S&amp;S 5 V</t>
+          <t>Citroën ë-C3 Eléctrico Max</t>
         </is>
       </c>
       <c r="F19" t="n">
@@ -1304,7 +1304,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>N1</t>
+          <t>M1</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1327,7 +1327,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>5937LLV</t>
+          <t>4450LLV</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1337,7 +1337,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>PEUGEOT Partner Premium Standard 600kg BlueHDi 100 S&amp;S 5 V</t>
+          <t>VOLKSWAGEN MULTIVAN 2.0TDI 198 PREMIUM 4M DSG</t>
         </is>
       </c>
       <c r="F20" t="n">
@@ -1350,7 +1350,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>N1</t>
+          <t>M1</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1373,7 +1373,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>6997LLV</t>
+          <t>4926LMS</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1383,7 +1383,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>PEUGEOT PARTNER 1.5 HDI 98 CV</t>
+          <t>PEUGEOT Partner Premium Standard 600kg BlueHDi 100 S&amp;S 5 V</t>
         </is>
       </c>
       <c r="F21" t="n">
@@ -1401,7 +1401,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>excel</t>
+          <t>extraccion</t>
         </is>
       </c>
       <c r="J21" t="inlineStr"/>
@@ -1419,7 +1419,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>9377LMG</t>
+          <t>5937LLV</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1429,7 +1429,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>PEUGEOT PARTNER 1.5 HDI 98 CV</t>
+          <t>PEUGEOT Partner Premium Standard 600kg BlueHDi 100 S&amp;S 5 V</t>
         </is>
       </c>
       <c r="F22" t="n">
@@ -1447,7 +1447,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>excel</t>
+          <t>extraccion</t>
         </is>
       </c>
       <c r="J22" t="inlineStr"/>
@@ -1465,7 +1465,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>9504LDD</t>
+          <t>6997LLV</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1475,7 +1475,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>OPEL GRANDLAND X</t>
+          <t>PEUGEOT PARTNER 1.5 HDI 98 CV</t>
         </is>
       </c>
       <c r="F23" t="n">
@@ -1488,12 +1488,12 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>M1</t>
+          <t>N1</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>extraccion</t>
+          <t>excel</t>
         </is>
       </c>
       <c r="J23" t="inlineStr"/>
@@ -1511,21 +1511,21 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2717MXG</t>
+          <t>8896LLB</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Nuevo (alta)</t>
+          <t>Sustituido (baja)</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>RENAULT KANGOO FURGON E-TECH 100% ELECTRIC</t>
+          <t>RENAULT KADJAR 4*4 1.8 DCI 150 CV</t>
         </is>
       </c>
       <c r="F24" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
@@ -1534,12 +1534,12 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>N1</t>
+          <t>M1</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>extraccion</t>
+          <t>excel</t>
         </is>
       </c>
       <c r="J24" t="inlineStr"/>
@@ -1557,21 +1557,21 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2732MWP</t>
+          <t>9504LDD</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Nuevo (alta)</t>
+          <t>Sustituido (baja)</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>CITROËN ë-C3 Eléctrico Max</t>
+          <t>OPEL GRANDLAND X</t>
         </is>
       </c>
       <c r="F25" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
@@ -1603,7 +1603,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2788MXG</t>
+          <t>2704MXG</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1649,7 +1649,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>5360MXF</t>
+          <t>2717MXG</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1695,7 +1695,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>6028MWV</t>
+          <t>2732MWP</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1741,7 +1741,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>6046MWV</t>
+          <t>2788MXG</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1751,7 +1751,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>CITROËN ë-C3 Eléctrico Max</t>
+          <t>RENAULT KANGOO FURGON E-TECH 100% ELECTRIC</t>
         </is>
       </c>
       <c r="F29" t="n">
@@ -1764,7 +1764,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>M1</t>
+          <t>N1</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -1787,7 +1787,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>6055MWV</t>
+          <t>5360MXF</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1797,7 +1797,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>CITROËN ë-C3 Eléctrico Max</t>
+          <t>RENAULT KANGOO FURGON E-TECH 100% ELECTRIC</t>
         </is>
       </c>
       <c r="F30" t="n">
@@ -1810,7 +1810,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>M1</t>
+          <t>N1</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -1833,7 +1833,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>6087MWV</t>
+          <t>6028MWV</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1879,7 +1879,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>6102MWV</t>
+          <t>6046MWV</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1925,7 +1925,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>6271MXF</t>
+          <t>6055MWV</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1935,7 +1935,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>RENAULT KANGOO FURGON E-TECH 100% ELECTRIC</t>
+          <t>CITROËN ë-C3 Eléctrico Max</t>
         </is>
       </c>
       <c r="F33" t="n">
@@ -1948,7 +1948,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>N1</t>
+          <t>M1</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -1971,7 +1971,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>9049MWN</t>
+          <t>6271MXF</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1981,7 +1981,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>CITROEN Ë-C3 ELÉCTRICO MAX</t>
+          <t>RENAULT KANGOO FURGON E-TECH 100% ELECTRIC</t>
         </is>
       </c>
       <c r="F34" t="n">
@@ -1994,12 +1994,12 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>M1</t>
+          <t>N1</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>excel</t>
+          <t>extraccion</t>
         </is>
       </c>
       <c r="J34" t="inlineStr"/>
@@ -2017,17 +2017,17 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>0894LKM</t>
+          <t>6370MXF</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Sustituido (baja)</t>
+          <t>Nuevo (alta)</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>SEAT León 1.6 Tdi 85kw (115cv) St&amp;sp Style</t>
+          <t>RENAULT KANGOO FURGON E-TECH 100% ELECTRIC</t>
         </is>
       </c>
       <c r="F35" t="n">
@@ -2040,7 +2040,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>M1</t>
+          <t>N1</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -2048,11 +2048,7 @@
           <t>extraccion</t>
         </is>
       </c>
-      <c r="J35" t="inlineStr">
-        <is>
-          <t>R2 Posesión: falta la fecha de salida; R9 Salida: no consta la fecha de salida</t>
-        </is>
-      </c>
+      <c r="J35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2067,7 +2063,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>0426KHR</t>
+          <t>0894LKM</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -2077,11 +2073,11 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>OPEL CORSA</t>
+          <t>SEAT León 1.6 Tdi 85kw (115cv) St&amp;sp Style</t>
         </is>
       </c>
       <c r="F36" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
@@ -2098,7 +2094,11 @@
           <t>extraccion</t>
         </is>
       </c>
-      <c r="J36" t="inlineStr"/>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>R2 Posesión: falta la fecha de salida; R9 Salida: no consta la fecha de salida</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2113,7 +2113,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>2096LKP</t>
+          <t>0426KHR</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -2123,7 +2123,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>RENAULT KADJAR 1.5 DCI 115 CV</t>
+          <t>OPEL CORSA</t>
         </is>
       </c>
       <c r="F37" t="n">
@@ -2141,7 +2141,7 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>excel</t>
+          <t>extraccion</t>
         </is>
       </c>
       <c r="J37" t="inlineStr"/>
@@ -2159,7 +2159,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>4450LLV</t>
+          <t>2096LKP</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -2169,7 +2169,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>VOLKSWAGEN MULTIVAN 2.0TDI 198 PREMIUM 4M DSG</t>
+          <t>RENAULT KADJAR 1.5 DCI 115 CV</t>
         </is>
       </c>
       <c r="F38" t="n">
@@ -2187,7 +2187,7 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>extraccion</t>
+          <t>excel</t>
         </is>
       </c>
       <c r="J38" t="inlineStr"/>
@@ -2297,7 +2297,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>8896LLB</t>
+          <t>9377LMG</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -2307,7 +2307,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>RENAULT KADJAR 4*4 1.8 DCI 150 CV</t>
+          <t>PEUGEOT PARTNER 1.5 HDI 98 CV</t>
         </is>
       </c>
       <c r="F41" t="n">
@@ -2320,7 +2320,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>M1</t>
+          <t>N1</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -4751,7 +4751,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>0679MWF</t>
+          <t>3256MXH</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -4761,7 +4761,7 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>NISSAN TOWNSTAR</t>
+          <t>RENAULT KANGOO VAN E-TECH ELECTRIC</t>
         </is>
       </c>
       <c r="F94" t="n">
@@ -4981,17 +4981,17 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>8496MXG</t>
+          <t>5918LLV</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Nuevo (alta)</t>
+          <t>Sustituido (baja)</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>RENAULT KANGOO FURGON E-TECH 100% ELECTRIC</t>
+          <t>PEUGEOT PARTNER</t>
         </is>
       </c>
       <c r="F99" t="n">
@@ -5027,7 +5027,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>5918LLV</t>
+          <t>9276LMB</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -5037,7 +5037,7 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>PEUGEOT PARTNER</t>
+          <t>SEAT Arona 1.6 Tdi 70kw (95cv) Style Ecomotive</t>
         </is>
       </c>
       <c r="F100" t="n">
@@ -5050,7 +5050,7 @@
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>N1</t>
+          <t>M1</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
@@ -5073,7 +5073,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>9276LMB</t>
+          <t>9305LMG</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -5083,7 +5083,7 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>SEAT Arona 1.6 Tdi 70kw (95cv) Style Ecomotive</t>
+          <t>PEUGEOT PARTNER ERKE</t>
         </is>
       </c>
       <c r="F101" t="n">
@@ -5096,7 +5096,7 @@
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>M1</t>
+          <t>N1</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
@@ -5119,21 +5119,21 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>9305LMG</t>
+          <t>0602KHK</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Sustituido (baja)</t>
+          <t>Nuevo (alta)</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>PEUGEOT PARTNER ERKE</t>
+          <t>RENAULT ZOE INTENS 40 R90 5P</t>
         </is>
       </c>
       <c r="F102" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G102" t="inlineStr">
         <is>
@@ -5142,7 +5142,7 @@
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>N1</t>
+          <t>M1</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
@@ -5165,7 +5165,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>0602KHK</t>
+          <t>0679MWF</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -5175,7 +5175,7 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>RENAULT ZOE INTENS 40 R90 5P</t>
+          <t>NISSAN TOWNSTAR</t>
         </is>
       </c>
       <c r="F103" t="n">
@@ -5188,12 +5188,12 @@
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>M1</t>
+          <t>N1</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>extraccion</t>
+          <t>excel</t>
         </is>
       </c>
       <c r="J103" t="inlineStr"/>
@@ -5211,7 +5211,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>3256MXH</t>
+          <t>6109MWV</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -5221,7 +5221,7 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>RENAULT KANGOO VAN E-TECH ELECTRIC</t>
+          <t>CITROEN Ë-C3 ELÉCTRICO MAX</t>
         </is>
       </c>
       <c r="F104" t="n">
@@ -5234,7 +5234,7 @@
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>N1</t>
+          <t>M1</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">
@@ -5257,7 +5257,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>6109MWV</t>
+          <t>6125MWV</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -5267,7 +5267,7 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>CITROEN Ë-C3 ELÉCTRICO MAX</t>
+          <t>Citroën ë-C3 Eléctrico Max</t>
         </is>
       </c>
       <c r="F105" t="n">
@@ -5285,7 +5285,7 @@
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>excel</t>
+          <t>extraccion</t>
         </is>
       </c>
       <c r="J105" t="inlineStr"/>
@@ -5303,7 +5303,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>6125MWV</t>
+          <t>6126MWV</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -5349,7 +5349,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>6126MWV</t>
+          <t>8249MXG</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -5359,7 +5359,7 @@
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>Citroën ë-C3 Eléctrico Max</t>
+          <t>RENAULT KANGOO FURGON E-TECH 100% ELECTRIC</t>
         </is>
       </c>
       <c r="F107" t="n">
@@ -5372,7 +5372,7 @@
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>M1</t>
+          <t>N1</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
@@ -5395,7 +5395,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>8249MXG</t>
+          <t>8387MXG</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -5441,7 +5441,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>8387MXG</t>
+          <t>8392MXG</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -5487,7 +5487,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>8392MXG</t>
+          <t>8436MXG</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -5533,7 +5533,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>8436MXG</t>
+          <t>8496MXG</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -6223,7 +6223,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>6033MWV</t>
+          <t>5665MWP</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
@@ -6269,7 +6269,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>6037MWV</t>
+          <t>6033MWV</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
@@ -6315,7 +6315,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>8628MWT</t>
+          <t>6037MWV</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
@@ -6325,7 +6325,7 @@
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>RENAULT KANGOO VAN E-TECH ELECTRIC</t>
+          <t>Citroën ë-C3 Eléctrico Max</t>
         </is>
       </c>
       <c r="F128" t="n">
@@ -6338,12 +6338,12 @@
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>N1</t>
+          <t>M1</t>
         </is>
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t>excel</t>
+          <t>extraccion</t>
         </is>
       </c>
       <c r="J128" t="inlineStr"/>
@@ -6361,7 +6361,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>8634MWT</t>
+          <t>8628MWT</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
@@ -6371,7 +6371,7 @@
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>RENAULT KANGOO FURGON E-TECH 100% ELECTRIC</t>
+          <t>RENAULT KANGOO VAN E-TECH ELECTRIC</t>
         </is>
       </c>
       <c r="F129" t="n">
@@ -6389,7 +6389,7 @@
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>extraccion</t>
+          <t>excel</t>
         </is>
       </c>
       <c r="J129" t="inlineStr"/>
@@ -6407,7 +6407,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>8658MWT</t>
+          <t>8634MWT</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -6453,17 +6453,17 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>7399LLP</t>
+          <t>8658MWT</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>Sustituido (baja)</t>
+          <t>Nuevo (alta)</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>RENAULT MASTER L2H2 2.3 DCI 135 CV</t>
+          <t>RENAULT KANGOO FURGON E-TECH 100% ELECTRIC</t>
         </is>
       </c>
       <c r="F131" t="n">
@@ -6481,7 +6481,7 @@
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>excel</t>
+          <t>extraccion</t>
         </is>
       </c>
       <c r="J131" t="inlineStr"/>
@@ -6499,7 +6499,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>9369LMG</t>
+          <t>2517LSG</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
@@ -6509,7 +6509,7 @@
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>PEUGEOT PARTNER 1.5 HDI 98 CV</t>
+          <t>DACIA SANDERO STEPWAY ECO 100 CV</t>
         </is>
       </c>
       <c r="F132" t="n">
@@ -6522,7 +6522,7 @@
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>N1</t>
+          <t>M1</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
@@ -6545,21 +6545,21 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>0682MWF</t>
+          <t>7399LLP</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>Nuevo (alta)</t>
+          <t>Sustituido (baja)</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>NISSAN Townstar Furgon 2 plazas 45kWh - 90kW (120CV) Comfort</t>
+          <t>RENAULT MASTER L2H2 2.3 DCI 135 CV</t>
         </is>
       </c>
       <c r="F133" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G133" t="inlineStr">
         <is>
@@ -6573,7 +6573,7 @@
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>extraccion</t>
+          <t>excel</t>
         </is>
       </c>
       <c r="J133" t="inlineStr"/>
@@ -6591,21 +6591,21 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>5665MWP</t>
+          <t>9369LMG</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>Nuevo (alta)</t>
+          <t>Sustituido (baja)</t>
         </is>
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>Citroën ë-C3 Eléctrico Max</t>
+          <t>PEUGEOT PARTNER 1.5 HDI 98 CV</t>
         </is>
       </c>
       <c r="F134" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G134" t="inlineStr">
         <is>
@@ -6614,12 +6614,12 @@
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>M1</t>
+          <t>N1</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>extraccion</t>
+          <t>excel</t>
         </is>
       </c>
       <c r="J134" t="inlineStr"/>
@@ -6637,7 +6637,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>6005MWV</t>
+          <t>0682MWF</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
@@ -6647,7 +6647,7 @@
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>CITROËN ë-C3 Eléctrico Max</t>
+          <t>NISSAN Townstar Furgon 2 plazas 45kWh - 90kW (120CV) Comfort</t>
         </is>
       </c>
       <c r="F135" t="n">
@@ -6660,7 +6660,7 @@
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>M1</t>
+          <t>N1</t>
         </is>
       </c>
       <c r="I135" t="inlineStr">
@@ -6683,7 +6683,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>6019MWV</t>
+          <t>6005MWV</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
@@ -6693,7 +6693,7 @@
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>CITROEN Ë-C3 ELÉCTRICO MAX</t>
+          <t>CITROËN ë-C3 Eléctrico Max</t>
         </is>
       </c>
       <c r="F136" t="n">
@@ -6711,7 +6711,7 @@
       </c>
       <c r="I136" t="inlineStr">
         <is>
-          <t>excel</t>
+          <t>extraccion</t>
         </is>
       </c>
       <c r="J136" t="inlineStr"/>
@@ -6729,7 +6729,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>6022MWV</t>
+          <t>6019MWV</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
@@ -6739,7 +6739,7 @@
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>Citroën ë-C3 Eléctrico Max</t>
+          <t>CITROEN Ë-C3 ELÉCTRICO MAX</t>
         </is>
       </c>
       <c r="F137" t="n">
@@ -6757,7 +6757,7 @@
       </c>
       <c r="I137" t="inlineStr">
         <is>
-          <t>extraccion</t>
+          <t>excel</t>
         </is>
       </c>
       <c r="J137" t="inlineStr"/>
@@ -6775,7 +6775,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>8626MWT</t>
+          <t>6022MWV</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
@@ -6785,7 +6785,7 @@
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>RENAULT KANGOO FURGON E-TECH 100% ELECTRIC</t>
+          <t>Citroën ë-C3 Eléctrico Max</t>
         </is>
       </c>
       <c r="F138" t="n">
@@ -6798,7 +6798,7 @@
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>N1</t>
+          <t>M1</t>
         </is>
       </c>
       <c r="I138" t="inlineStr">
@@ -6821,7 +6821,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>8627MWT</t>
+          <t>8626MWT</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
@@ -6867,7 +6867,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>8636MWT</t>
+          <t>8627MWT</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
@@ -6913,7 +6913,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>8637MWT</t>
+          <t>8636MWT</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
@@ -6959,7 +6959,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>8640MWT</t>
+          <t>8637MWT</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
@@ -6969,7 +6969,7 @@
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>RENAULT KANGOO VAN E-TECH ELECTRIC</t>
+          <t>RENAULT KANGOO FURGON E-TECH 100% ELECTRIC</t>
         </is>
       </c>
       <c r="F142" t="n">
@@ -6987,7 +6987,7 @@
       </c>
       <c r="I142" t="inlineStr">
         <is>
-          <t>excel</t>
+          <t>extraccion</t>
         </is>
       </c>
       <c r="J142" t="inlineStr"/>
@@ -7005,7 +7005,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>8642MWT</t>
+          <t>8640MWT</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
@@ -7051,7 +7051,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>8644MWT</t>
+          <t>8642MWT</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
@@ -7097,7 +7097,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>8647MWT</t>
+          <t>8644MWT</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
@@ -7107,7 +7107,7 @@
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>RENAULT KANGOO FURGON E-TECH 100% ELECTRIC</t>
+          <t>RENAULT KANGOO VAN E-TECH ELECTRIC</t>
         </is>
       </c>
       <c r="F145" t="n">
@@ -7125,7 +7125,7 @@
       </c>
       <c r="I145" t="inlineStr">
         <is>
-          <t>extraccion</t>
+          <t>excel</t>
         </is>
       </c>
       <c r="J145" t="inlineStr"/>
@@ -7143,7 +7143,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>8651MWT</t>
+          <t>8647MWT</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
@@ -7189,21 +7189,21 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>2517LSG</t>
+          <t>8651MWT</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>Sustituido (baja)</t>
+          <t>Nuevo (alta)</t>
         </is>
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>DACIA SANDERO STEPWAY ECO 100 CV</t>
+          <t>RENAULT KANGOO FURGON E-TECH 100% ELECTRIC</t>
         </is>
       </c>
       <c r="F147" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G147" t="inlineStr">
         <is>
@@ -7212,12 +7212,12 @@
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>M1</t>
+          <t>N1</t>
         </is>
       </c>
       <c r="I147" t="inlineStr">
         <is>
-          <t>excel</t>
+          <t>extraccion</t>
         </is>
       </c>
       <c r="J147" t="inlineStr"/>
@@ -10101,7 +10101,7 @@
         </is>
       </c>
       <c r="F210" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G210" t="inlineStr">
         <is>
@@ -10409,7 +10409,7 @@
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>3189LLY</t>
+          <t>6744LLV</t>
         </is>
       </c>
       <c r="D217" t="inlineStr">
@@ -10455,7 +10455,7 @@
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>3200LLY</t>
+          <t>9416LMG</t>
         </is>
       </c>
       <c r="D218" t="inlineStr">
@@ -10501,7 +10501,7 @@
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>5941LLV</t>
+          <t>0722KVP</t>
         </is>
       </c>
       <c r="D219" t="inlineStr">
@@ -10511,11 +10511,11 @@
       </c>
       <c r="E219" t="inlineStr">
         <is>
-          <t>PEUGEOT PARTNER 1.5 HDI 98 CV</t>
+          <t>OPEL ASTRA 1.6 CDTI 110 CV</t>
         </is>
       </c>
       <c r="F219" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G219" t="inlineStr">
         <is>
@@ -10524,7 +10524,7 @@
       </c>
       <c r="H219" t="inlineStr">
         <is>
-          <t>N1</t>
+          <t>M1</t>
         </is>
       </c>
       <c r="I219" t="inlineStr">
@@ -10547,7 +10547,7 @@
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>6744LLV</t>
+          <t>0841KWW</t>
         </is>
       </c>
       <c r="D220" t="inlineStr">
@@ -10557,11 +10557,11 @@
       </c>
       <c r="E220" t="inlineStr">
         <is>
-          <t>PEUGEOT PARTNER 1.5 HDI 98 CV</t>
+          <t>OPEL ASTRA 1.6 CDTI 110 CV</t>
         </is>
       </c>
       <c r="F220" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G220" t="inlineStr">
         <is>
@@ -10570,7 +10570,7 @@
       </c>
       <c r="H220" t="inlineStr">
         <is>
-          <t>N1</t>
+          <t>M1</t>
         </is>
       </c>
       <c r="I220" t="inlineStr">
@@ -10593,7 +10593,7 @@
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>9197LKX</t>
+          <t>3189LLY</t>
         </is>
       </c>
       <c r="D221" t="inlineStr">
@@ -10603,11 +10603,11 @@
       </c>
       <c r="E221" t="inlineStr">
         <is>
-          <t>VOLKSWAGEN CADDY 4*4 2.0 TDI 122 CV</t>
+          <t>PEUGEOT PARTNER 1.5 HDI 98 CV</t>
         </is>
       </c>
       <c r="F221" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G221" t="inlineStr">
         <is>
@@ -10639,7 +10639,7 @@
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>9275LMG</t>
+          <t>3200LLY</t>
         </is>
       </c>
       <c r="D222" t="inlineStr">
@@ -10653,7 +10653,7 @@
         </is>
       </c>
       <c r="F222" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G222" t="inlineStr">
         <is>
@@ -10685,7 +10685,7 @@
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>9416LMG</t>
+          <t>5478LLD</t>
         </is>
       </c>
       <c r="D223" t="inlineStr">
@@ -10695,11 +10695,11 @@
       </c>
       <c r="E223" t="inlineStr">
         <is>
-          <t>PEUGEOT PARTNER 1.5 HDI 98 CV</t>
+          <t>VOLKSWAGEN CADDY 4*4 2.0 TDI 122 CV KOMBI</t>
         </is>
       </c>
       <c r="F223" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G223" t="inlineStr">
         <is>
@@ -10708,7 +10708,7 @@
       </c>
       <c r="H223" t="inlineStr">
         <is>
-          <t>N1</t>
+          <t>M1</t>
         </is>
       </c>
       <c r="I223" t="inlineStr">
@@ -10731,7 +10731,7 @@
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>0722KVP</t>
+          <t>9197LKX</t>
         </is>
       </c>
       <c r="D224" t="inlineStr">
@@ -10741,7 +10741,7 @@
       </c>
       <c r="E224" t="inlineStr">
         <is>
-          <t>OPEL ASTRA 1.6 CDTI 110 CV</t>
+          <t>VOLKSWAGEN CADDY 4*4 2.0 TDI 122 CV</t>
         </is>
       </c>
       <c r="F224" t="n">
@@ -10754,7 +10754,7 @@
       </c>
       <c r="H224" t="inlineStr">
         <is>
-          <t>M1</t>
+          <t>N1</t>
         </is>
       </c>
       <c r="I224" t="inlineStr">
@@ -10777,7 +10777,7 @@
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>0841KWW</t>
+          <t>9275LMG</t>
         </is>
       </c>
       <c r="D225" t="inlineStr">
@@ -10787,7 +10787,7 @@
       </c>
       <c r="E225" t="inlineStr">
         <is>
-          <t>OPEL ASTRA 1.6 CDTI 110 CV</t>
+          <t>PEUGEOT PARTNER 1.5 HDI 98 CV</t>
         </is>
       </c>
       <c r="F225" t="n">
@@ -10800,7 +10800,7 @@
       </c>
       <c r="H225" t="inlineStr">
         <is>
-          <t>M1</t>
+          <t>N1</t>
         </is>
       </c>
       <c r="I225" t="inlineStr">
@@ -10823,7 +10823,7 @@
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>5478LLD</t>
+          <t>9471LKC</t>
         </is>
       </c>
       <c r="D226" t="inlineStr">
@@ -10833,7 +10833,7 @@
       </c>
       <c r="E226" t="inlineStr">
         <is>
-          <t>VOLKSWAGEN CADDY 4*4 2.0 TDI 122 CV KOMBI</t>
+          <t>SEAT ARONA 1.6 TDI 95 CV</t>
         </is>
       </c>
       <c r="F226" t="n">
@@ -10859,27 +10859,27 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>1400</t>
+          <t>1490</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>EGEVASA</t>
+          <t>EMPRESA MIXTA CALPE</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>9471LKC</t>
+          <t>7151MXV</t>
         </is>
       </c>
       <c r="D227" t="inlineStr">
         <is>
-          <t>Sustituido (baja)</t>
+          <t>Nuevo (alta)</t>
         </is>
       </c>
       <c r="E227" t="inlineStr">
         <is>
-          <t>SEAT ARONA 1.6 TDI 95 CV</t>
+          <t>RENAULT KANGOO FURGON E-TECH 100% ELECTRIC</t>
         </is>
       </c>
       <c r="F227" t="n">
@@ -10892,12 +10892,12 @@
       </c>
       <c r="H227" t="inlineStr">
         <is>
-          <t>M1</t>
+          <t>N1</t>
         </is>
       </c>
       <c r="I227" t="inlineStr">
         <is>
-          <t>excel</t>
+          <t>extraccion</t>
         </is>
       </c>
       <c r="J227" t="inlineStr"/>
@@ -10915,17 +10915,17 @@
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>7151MXV</t>
+          <t>9850JTR</t>
         </is>
       </c>
       <c r="D228" t="inlineStr">
         <is>
-          <t>Nuevo (alta)</t>
+          <t>Sustituido (baja)</t>
         </is>
       </c>
       <c r="E228" t="inlineStr">
         <is>
-          <t>RENAULT KANGOO FURGON E-TECH 100% ELECTRIC</t>
+          <t>Opel Movano 2.3 Cdti 130 L3H1 R 3.5t Hd Bascul. Ace</t>
         </is>
       </c>
       <c r="F228" t="n">
@@ -11237,7 +11237,7 @@
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>8994MSH</t>
+          <t>8625MWT</t>
         </is>
       </c>
       <c r="D235" t="inlineStr">
@@ -11247,7 +11247,7 @@
       </c>
       <c r="E235" t="inlineStr">
         <is>
-          <t>NISSAN TOWNSTAR FURGÓN 2 PLAZAS 45KWH - 90KW (120CV) L1 COMFORT</t>
+          <t>RENAULT KANGOO FURGON E-TECH 100% ELECTRIC</t>
         </is>
       </c>
       <c r="F235" t="n">
@@ -11283,7 +11283,7 @@
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>8999MSH</t>
+          <t>8994MSH</t>
         </is>
       </c>
       <c r="D236" t="inlineStr">
@@ -11293,7 +11293,7 @@
       </c>
       <c r="E236" t="inlineStr">
         <is>
-          <t>NISSAN TOWNSTAR</t>
+          <t>NISSAN TOWNSTAR FURGÓN 2 PLAZAS 45KWH - 90KW (120CV) L1 COMFORT</t>
         </is>
       </c>
       <c r="F236" t="n">
@@ -11311,7 +11311,7 @@
       </c>
       <c r="I236" t="inlineStr">
         <is>
-          <t>excel</t>
+          <t>extraccion</t>
         </is>
       </c>
       <c r="J236" t="inlineStr"/>
@@ -11329,17 +11329,17 @@
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>0019LLR</t>
+          <t>8998MSH</t>
         </is>
       </c>
       <c r="D237" t="inlineStr">
         <is>
-          <t>Sustituido (baja)</t>
+          <t>Nuevo (alta)</t>
         </is>
       </c>
       <c r="E237" t="inlineStr">
         <is>
-          <t>SEAT LEON</t>
+          <t>NISSAN TOWNSTAR</t>
         </is>
       </c>
       <c r="F237" t="n">
@@ -11352,12 +11352,12 @@
       </c>
       <c r="H237" t="inlineStr">
         <is>
-          <t>M1</t>
+          <t>N1</t>
         </is>
       </c>
       <c r="I237" t="inlineStr">
         <is>
-          <t>extraccion</t>
+          <t>excel</t>
         </is>
       </c>
       <c r="J237" t="inlineStr"/>
@@ -11375,7 +11375,7 @@
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>1188JZF</t>
+          <t>0019LLR</t>
         </is>
       </c>
       <c r="D238" t="inlineStr">
@@ -11385,7 +11385,7 @@
       </c>
       <c r="E238" t="inlineStr">
         <is>
-          <t>TOYOTA INDUST. Hilux 2.4 D-4d Cabina Doble</t>
+          <t>SEAT LEON</t>
         </is>
       </c>
       <c r="F238" t="n">
@@ -11398,7 +11398,7 @@
       </c>
       <c r="H238" t="inlineStr">
         <is>
-          <t>N1</t>
+          <t>M1</t>
         </is>
       </c>
       <c r="I238" t="inlineStr">
@@ -11421,7 +11421,7 @@
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>1192LPK</t>
+          <t>1188JZF</t>
         </is>
       </c>
       <c r="D239" t="inlineStr">
@@ -11431,7 +11431,7 @@
       </c>
       <c r="E239" t="inlineStr">
         <is>
-          <t>SEAT ARONA 1.6 TDI 95 CV</t>
+          <t>TOYOTA INDUST. Hilux 2.4 D-4d Cabina Doble</t>
         </is>
       </c>
       <c r="F239" t="n">
@@ -11444,12 +11444,12 @@
       </c>
       <c r="H239" t="inlineStr">
         <is>
-          <t>M1</t>
+          <t>N1</t>
         </is>
       </c>
       <c r="I239" t="inlineStr">
         <is>
-          <t>excel</t>
+          <t>extraccion</t>
         </is>
       </c>
       <c r="J239" t="inlineStr"/>
@@ -11559,7 +11559,7 @@
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>6756LLV</t>
+          <t>5949LLV</t>
         </is>
       </c>
       <c r="D242" t="inlineStr">
@@ -11569,7 +11569,7 @@
       </c>
       <c r="E242" t="inlineStr">
         <is>
-          <t>PEUGEOT Partner Premium Standard 600kg BlueHDi 100 S&amp;S 5 V</t>
+          <t>PEUGEOT PARTNER</t>
         </is>
       </c>
       <c r="F242" t="n">
@@ -11605,21 +11605,21 @@
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>6847MWL</t>
+          <t>6756LLV</t>
         </is>
       </c>
       <c r="D243" t="inlineStr">
         <is>
-          <t>Nuevo (alta)</t>
+          <t>Sustituido (baja)</t>
         </is>
       </c>
       <c r="E243" t="inlineStr">
         <is>
-          <t>NISSAN Townstar Furgon 2 plazas 45kWh - 90kW (120CV) Comfort</t>
+          <t>PEUGEOT Partner Premium Standard 600kg BlueHDi 100 S&amp;S 5 V</t>
         </is>
       </c>
       <c r="F243" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G243" t="inlineStr">
         <is>
@@ -11651,21 +11651,21 @@
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>8601MWT</t>
+          <t>7995LKS</t>
         </is>
       </c>
       <c r="D244" t="inlineStr">
         <is>
-          <t>Nuevo (alta)</t>
+          <t>Sustituido (baja)</t>
         </is>
       </c>
       <c r="E244" t="inlineStr">
         <is>
-          <t>RENAULT KANGOO FURGON E-TECH 100% ELECTRIC</t>
+          <t>RENAULT KADJAR 4*4 1.8 DCI 150 CV</t>
         </is>
       </c>
       <c r="F244" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G244" t="inlineStr">
         <is>
@@ -11674,12 +11674,12 @@
       </c>
       <c r="H244" t="inlineStr">
         <is>
-          <t>N1</t>
+          <t>M1</t>
         </is>
       </c>
       <c r="I244" t="inlineStr">
         <is>
-          <t>extraccion</t>
+          <t>excel</t>
         </is>
       </c>
       <c r="J244" t="inlineStr"/>
@@ -11697,7 +11697,7 @@
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>8603MWT</t>
+          <t>1066MWL</t>
         </is>
       </c>
       <c r="D245" t="inlineStr">
@@ -11707,7 +11707,7 @@
       </c>
       <c r="E245" t="inlineStr">
         <is>
-          <t>RENAULT KANGOO FURGON E-TECH 100% ELECTRIC</t>
+          <t>CITROËN Berlingo Talla M BlueHDi 100 S&amp;S 6</t>
         </is>
       </c>
       <c r="F245" t="n">
@@ -11743,7 +11743,7 @@
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>8606MWT</t>
+          <t>6847MWL</t>
         </is>
       </c>
       <c r="D246" t="inlineStr">
@@ -11753,7 +11753,7 @@
       </c>
       <c r="E246" t="inlineStr">
         <is>
-          <t>RENAULT KANGOO FURGON E-TECH 100% ELECTRIC</t>
+          <t>NISSAN Townstar Furgon 2 plazas 45kWh - 90kW (120CV) Comfort</t>
         </is>
       </c>
       <c r="F246" t="n">
@@ -11789,7 +11789,7 @@
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>8616MWT</t>
+          <t>8601MWT</t>
         </is>
       </c>
       <c r="D247" t="inlineStr">
@@ -11835,7 +11835,7 @@
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>8617MWT</t>
+          <t>8603MWT</t>
         </is>
       </c>
       <c r="D248" t="inlineStr">
@@ -11881,7 +11881,7 @@
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>8618MWT</t>
+          <t>8606MWT</t>
         </is>
       </c>
       <c r="D249" t="inlineStr">
@@ -11927,7 +11927,7 @@
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>8619MWT</t>
+          <t>8616MWT</t>
         </is>
       </c>
       <c r="D250" t="inlineStr">
@@ -11973,7 +11973,7 @@
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>8624MWT</t>
+          <t>8617MWT</t>
         </is>
       </c>
       <c r="D251" t="inlineStr">
@@ -12019,7 +12019,7 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>8625MWT</t>
+          <t>8618MWT</t>
         </is>
       </c>
       <c r="D252" t="inlineStr">
@@ -12065,7 +12065,7 @@
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>8998MSH</t>
+          <t>8619MWT</t>
         </is>
       </c>
       <c r="D253" t="inlineStr">
@@ -12075,7 +12075,7 @@
       </c>
       <c r="E253" t="inlineStr">
         <is>
-          <t>NISSAN TOWNSTAR</t>
+          <t>RENAULT KANGOO FURGON E-TECH 100% ELECTRIC</t>
         </is>
       </c>
       <c r="F253" t="n">
@@ -12093,7 +12093,7 @@
       </c>
       <c r="I253" t="inlineStr">
         <is>
-          <t>excel</t>
+          <t>extraccion</t>
         </is>
       </c>
       <c r="J253" t="inlineStr"/>
@@ -12111,21 +12111,21 @@
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>4719KYS</t>
+          <t>8624MWT</t>
         </is>
       </c>
       <c r="D254" t="inlineStr">
         <is>
-          <t>Sustituido (baja)</t>
+          <t>Nuevo (alta)</t>
         </is>
       </c>
       <c r="E254" t="inlineStr">
         <is>
-          <t>VOLVO XC60</t>
+          <t>RENAULT KANGOO FURGON E-TECH 100% ELECTRIC</t>
         </is>
       </c>
       <c r="F254" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G254" t="inlineStr">
         <is>
@@ -12134,7 +12134,7 @@
       </c>
       <c r="H254" t="inlineStr">
         <is>
-          <t>M1</t>
+          <t>N1</t>
         </is>
       </c>
       <c r="I254" t="inlineStr">
@@ -12157,21 +12157,21 @@
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>5949LLV</t>
+          <t>8999MSH</t>
         </is>
       </c>
       <c r="D255" t="inlineStr">
         <is>
-          <t>Sustituido (baja)</t>
+          <t>Nuevo (alta)</t>
         </is>
       </c>
       <c r="E255" t="inlineStr">
         <is>
-          <t>PEUGEOT PARTNER</t>
+          <t>NISSAN TOWNSTAR</t>
         </is>
       </c>
       <c r="F255" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G255" t="inlineStr">
         <is>
@@ -12185,7 +12185,7 @@
       </c>
       <c r="I255" t="inlineStr">
         <is>
-          <t>extraccion</t>
+          <t>excel</t>
         </is>
       </c>
       <c r="J255" t="inlineStr"/>
@@ -12203,7 +12203,7 @@
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>6586KPD</t>
+          <t>4719KYS</t>
         </is>
       </c>
       <c r="D256" t="inlineStr">
@@ -12213,7 +12213,7 @@
       </c>
       <c r="E256" t="inlineStr">
         <is>
-          <t>OPEL COMBO</t>
+          <t>VOLVO XC60</t>
         </is>
       </c>
       <c r="F256" t="n">
@@ -12226,7 +12226,7 @@
       </c>
       <c r="H256" t="inlineStr">
         <is>
-          <t>N1</t>
+          <t>M1</t>
         </is>
       </c>
       <c r="I256" t="inlineStr">
@@ -12249,7 +12249,7 @@
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>7995LKS</t>
+          <t>6586KPD</t>
         </is>
       </c>
       <c r="D257" t="inlineStr">
@@ -12259,7 +12259,7 @@
       </c>
       <c r="E257" t="inlineStr">
         <is>
-          <t>RENAULT KADJAR 4*4 1.8 DCI 150 CV</t>
+          <t>OPEL COMBO</t>
         </is>
       </c>
       <c r="F257" t="n">
@@ -12272,12 +12272,12 @@
       </c>
       <c r="H257" t="inlineStr">
         <is>
-          <t>M1</t>
+          <t>N1</t>
         </is>
       </c>
       <c r="I257" t="inlineStr">
         <is>
-          <t>excel</t>
+          <t>extraccion</t>
         </is>
       </c>
       <c r="J257" t="inlineStr"/>

</xml_diff>